<commit_message>
add the rest of the local byelections for 2014-2016
</commit_message>
<xml_diff>
--- a/src/data/raw/2016_22_ოქტომბერი_განმეორებითი.xlsx
+++ b/src/data/raw/2016_22_ოქტომბერი_განმეორებითი.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23901"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Election portal data sets\Election results\შედეგები\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox (Personal)\My projects\Elections\ge_elections_dashboard\wireframe\observable_framework\elections_data\src\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F081E724-0455-4F96-BC3A-E7B38AAC0515}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1B99F6B-9ADF-4F23-826C-E1170BF6DE2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="w_20161022" sheetId="1" r:id="rId1"/>
+    <sheet name="კანდიდატები" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="85">
   <si>
     <t>მაჟორიტარული ოლქის N</t>
   </si>
@@ -142,17 +143,899 @@
   </si>
   <si>
     <t>vote_44</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>#</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>საოლქო საარჩევნო კომისიის დასახელება</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>მაჟორიტარული საარჩევნო ოლქი</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>კანდიდატის ნომერი</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>წარმდგენი</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>სახელი</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>გვარი</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>მარნეული</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>7. „</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">თამაზ მეჭიაური ერთიანი
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>საქართველოსთვის</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>”</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>ელდარ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>მუსტაფაევი</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">8. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">საარჩევნო ბლოკი </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>„</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>დავით თარხან</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">‐ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>მოურავი</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">ირმა ინაშვილი </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">‐ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>საქართველოს პატრიოტთა ალიანსი</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>გაერთიანებული ოპოზიცია</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>”</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>ალი</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>ისაევი</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>17. „</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>საქართველო</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>”</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>ომარ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>წამალაიძე</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>გურგენიშვილი</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">23. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">საარჩევნო ბლოკი </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>„</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">ჩვენები </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">‐ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">სახალხო
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>პარტია</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>”</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>თეონა</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>ქავთარია</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>41. „</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">ქართული ოცნება </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">‐ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">დემოკრატიული
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>საქართველო</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>”</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>თამაზ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>ნავერიანი</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">საარჩევნო ბლოკი </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>„</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">პაატა ბურჭულაძე </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">‐
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>სახელმწიფო ხალხისთვის</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>”</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>ისრაფილ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>ბაირამოვი</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">საარჩევნო ბლოკი </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>„</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">ნინო ბურჯანაძე </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">‐
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>დემოკრატიული მოძრაობა</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>”</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>ვეფხია</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">5. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">საარჩევნო ბლოკი </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>„</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">ერთიანი
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>ნაციონალური მოძრაობა</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>”</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>აკმამედ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>იმამკულიევი</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>ზუგდიდი</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>ბესიკ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>თოდუა</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">სანდრა
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>ელისაბედ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>რულოვს</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>ჯონი</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>ზარანდია</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>28. „</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">ზვიადის გზა </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">‐ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>უფლის სახელით</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>”</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>რამაზ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>ჩაჩიბაია</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>ირაკლი</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>ჩანგელია</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>ედიშერ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Sylfaen"/>
+        <family val="1"/>
+      </rPr>
+      <t>თოლორაია</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Sylfaen"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -160,7 +1043,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Sylfaen"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -168,12 +1051,34 @@
       <b/>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Sylfaen"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Sylfaen"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -186,8 +1091,13 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -210,11 +1120,39 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -223,9 +1161,57 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="ჩვეულებრივი" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -512,16 +1498,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AI5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" customWidth="1"/>
-    <col min="2" max="2" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.53515625" customWidth="1"/>
+    <col min="2" max="2" width="9.07421875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17" customWidth="1"/>
-    <col min="4" max="4" width="16.44140625" customWidth="1"/>
-    <col min="5" max="5" width="12.44140625" customWidth="1"/>
+    <col min="4" max="4" width="16.4609375" customWidth="1"/>
+    <col min="5" max="5" width="12.4609375" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="16.88671875" customWidth="1"/>
-    <col min="8" max="8" width="16.44140625" customWidth="1"/>
+    <col min="7" max="7" width="16.84375" customWidth="1"/>
+    <col min="8" max="8" width="16.4609375" customWidth="1"/>
     <col min="9" max="9" width="5" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="2" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="4" bestFit="1" customWidth="1"/>
@@ -537,7 +1523,7 @@
     <col min="35" max="35" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:35" ht="27" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -644,7 +1630,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.4">
       <c r="A2" s="2">
         <v>36</v>
       </c>
@@ -715,7 +1701,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
         <v>66</v>
       </c>
@@ -782,7 +1768,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <v>66</v>
       </c>
@@ -849,7 +1835,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>66</v>
       </c>
@@ -924,4 +1910,359 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B4F9B93-8EFD-4F8E-8F2A-65B7A9C73EF0}">
+  <dimension ref="A1:G15"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A1" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" s="17" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.9" x14ac:dyDescent="0.4">
+      <c r="A2" s="14">
+        <v>22</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="13">
+        <v>36</v>
+      </c>
+      <c r="D2" s="13">
+        <v>1</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="G2" s="18" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15.9" x14ac:dyDescent="0.4">
+      <c r="A3" s="14">
+        <v>22</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="5">
+        <v>36</v>
+      </c>
+      <c r="D3" s="11">
+        <v>3</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15.9" x14ac:dyDescent="0.4">
+      <c r="A4" s="15">
+        <v>22</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="4">
+        <v>36</v>
+      </c>
+      <c r="D4" s="7">
+        <v>5</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15.9" x14ac:dyDescent="0.4">
+      <c r="A5" s="15">
+        <v>22</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="4">
+        <v>36</v>
+      </c>
+      <c r="D5" s="7">
+        <v>7</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15.9" x14ac:dyDescent="0.4">
+      <c r="A6" s="14">
+        <v>22</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="5">
+        <v>36</v>
+      </c>
+      <c r="D6" s="11">
+        <v>8</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.9" x14ac:dyDescent="0.4">
+      <c r="A7" s="15">
+        <v>22</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="4">
+        <v>36</v>
+      </c>
+      <c r="D7" s="7">
+        <v>17</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15.9" x14ac:dyDescent="0.4">
+      <c r="A8" s="15">
+        <v>22</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="4">
+        <v>36</v>
+      </c>
+      <c r="D8" s="7">
+        <v>23</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15.9" x14ac:dyDescent="0.4">
+      <c r="A9" s="15">
+        <v>22</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="4">
+        <v>36</v>
+      </c>
+      <c r="D9" s="7">
+        <v>41</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15.9" x14ac:dyDescent="0.4">
+      <c r="A10" s="14">
+        <v>67</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="C10" s="5">
+        <v>66</v>
+      </c>
+      <c r="D10" s="11">
+        <v>1</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.9" x14ac:dyDescent="0.4">
+      <c r="A11" s="15">
+        <v>67</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C11" s="4">
+        <v>66</v>
+      </c>
+      <c r="D11" s="7">
+        <v>5</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15.9" x14ac:dyDescent="0.4">
+      <c r="A12" s="15">
+        <v>67</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C12" s="4">
+        <v>66</v>
+      </c>
+      <c r="D12" s="7">
+        <v>7</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15.9" x14ac:dyDescent="0.4">
+      <c r="A13" s="15">
+        <v>67</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" s="4">
+        <v>66</v>
+      </c>
+      <c r="D13" s="7">
+        <v>28</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15.9" x14ac:dyDescent="0.4">
+      <c r="A14" s="14">
+        <v>67</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="C14" s="5">
+        <v>66</v>
+      </c>
+      <c r="D14" s="11">
+        <v>8</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15.9" x14ac:dyDescent="0.4">
+      <c r="A15" s="15">
+        <v>67</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C15" s="4">
+        <v>66</v>
+      </c>
+      <c r="D15" s="7">
+        <v>41</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>84</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>